<commit_message>
fix: align spreadsheet handling with DPO reference
</commit_message>
<xml_diff>
--- a/docs/samples/sample_specification.xlsx
+++ b/docs/samples/sample_specification.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Техническое задание" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лист1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,36 +26,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00008B76"/>
+      <name val="Calibri"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00008B76"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,29 +56,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,290 +459,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="9.140000000000001" customWidth="1" min="1" max="1"/>
+    <col width="34.28" customWidth="1" min="2" max="2"/>
+    <col width="114.71" customWidth="1" min="3" max="3"/>
+    <col width="7.85" customWidth="1" min="4" max="4"/>
+    <col width="20.71" customWidth="1" min="5" max="5"/>
+    <col width="11.42" customWidth="1" min="6" max="6"/>
+    <col width="32.42" customWidth="1" min="7" max="7"/>
+    <col width="83.28" customWidth="1" min="8" max="8"/>
+    <col width="16.28" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ТЕХНИЧЕСКОЕ ЗАДАНИЕ</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Спецификация</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="80.25" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Характеристики</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Стоимость (долларов США/руб., c учетом НДС)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Срок поставки (рабочих дней)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Гарантия</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ссылки на ресурс, при наличии </t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Адрес поставки</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Предмет закупки</t>
-        </is>
+      <c r="A3" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Поставка ноутбуков</t>
+          <t>Ноутбук Альфа</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>RAM 16 ГБ; SSD 512 ГБ</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>24 месяца</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Москва</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Цель закупки</t>
-        </is>
+      <c r="A4" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Оснащение рабочих мест сотрудников</t>
+          <t>Ноутбук Бета</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>RAM 32 ГБ; SSD 1 ТБ</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>36 месяцев</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Москва</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Объём работ / поставки</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Поставка 5 ноутбуков без установки</t>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Общие требования:
+- Только поставка, без установки</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Срок выполнения</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>20 рабочих дней</t>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Блокирующие требования:
+- Не допускается восстановленное оборудование</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Критерии приёмки</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Соответствие количеству и заявленным характеристикам</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Описание</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Количество</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Ед. изм.</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Цена за единицу</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Стоимость</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Характеристики</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>Срок поставки</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Гарантия</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Адрес поставки</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Ссылка</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Ноутбук Альфа</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>RAM 16 ГБ; SSD 512 ГБ</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>24 месяца</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>Москва</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Ноутбук Бета</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>RAM 32 ГБ; SSD 1 ТБ</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>36 месяцев</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Москва</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Общие требования</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>• Только поставка, без установки</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Блокирующие требования</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>• Не допускается восстановленное оборудование</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Дополнительные условия</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>• Упаковка должна обеспечивать сохранность при транспортировке</t>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Дополнительные условия:
+- Упаковка должна обеспечивать сохранность при транспортировке</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="A20:M20"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>